<commit_message>
prg Sun Jun 14 04:31:29 PM CEST 2026
</commit_message>
<xml_diff>
--- a/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV06_pvgisampliado.xlsx
+++ b/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV06_pvgisampliado.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mi rrrr Real</t>
+          <t>alhori</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -853,16 +853,16 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1780945446828</v>
+        <v>1781116054277</v>
       </c>
       <c r="F2" t="n">
-        <v>36.66613004997789</v>
+        <v>37.12748581055218</v>
       </c>
       <c r="G2" t="n">
-        <v>-4.461177103172596</v>
+        <v>-3.220698684453964</v>
       </c>
       <c r="H2" t="n">
-        <v>-53.3438915840331</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>1.1</v>
@@ -930,17 +930,17 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>['-1,-3','-1,-2','-1,-1','-1,0','-1,1','0,-3','0,-2','0,-1','0,0','0,1']</t>
+          <t>['-1,-3','-1,-2','-1,-1','-1,0','-1,1','-1,2','0,-3','0,-2','0,1','0,2','0,-1','0,0']</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>[1,1,1,1,1,1,1,1,1,1,20,1,1,1,1,1]</t>
+          <t>[81,81,81,81,81,81,81,81,81,81,85,66,77,81,81,81]</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>{'type':'FeatureCollection','features':[{'type':'Feature','properties':{'area':'G2','block':'-1,-3'},'geometry':{'type':'Polygon','coordinates':[[[-4.46121023591994,36.666106716932475],[-4.461202881311809,36.66611464417448],[-4.4612176645495865,36.66612346877769],[-4.461225019157716,36.66611554153569],[-4.46121023591994,36.666106716932475]]]}},{'type':'Feature','properties':{'area':'G2','block':'-1,-2'},'geometry':{'type':'Polygon','coordinates':[[[-4.461202881311809,36.66611464417448],[-4.46119552670368,36.66612257141649],[-4.461210309941457,36.66613139601969],[-4.4612176645495865,36.66612346877769],[-4.461202881311809,36.66611464417448]]]}},{'type':'Feature','properties':{'area':'G2','block':'-1,-1'},'geometry':{'type':'Polygon','coordinates':[[[-4.46119552670368,36.66612257141649],[-4.461188172095549,36.66613049865849],[-4.461202955333326,36.6661393232617],[-4.461210309941457,36.66613139601969],[-4.46119552670368,36.66612257141649]]]}},{'type':'Feature','properties':{'area':'G2','block':'-1,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.461188172095549,36.66613049865849],[-4.46118081748742,36.66613842590049],[-4.461195600725197,36.666147250503705],[-4.461202955333326,36.6661393232617],[-4.461188172095549,36.66613049865849]]]}},{'type':'Feature','properties':{'area':'G2','block':'-1,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.46118081748742,36.66613842590049],[-4.461173462879289,36.6661463531425],[-4.461188246117066,36.66615517774571],[-4.461195600725197,36.666147250503705],[-4.46118081748742,36.66613842590049]]]}},{'type':'Feature','properties':{'area':'G2','block':'0,-3'},'geometry':{'type':'Polygon','coordinates':[[[-4.461195452682163,36.66609789232926],[-4.461188098074032,36.66610581957127],[-4.461202881311809,36.66611464417448],[-4.46121023591994,36.666106716932475],[-4.461195452682163,36.66609789232926]]]}},{'type':'Feature','properties':{'area':'G2','block':'0,-2'},'geometry':{'type':'Polygon','coordinates':[[[-4.461188098074032,36.66610581957127],[-4.461180743465903,36.666113746813274],[-4.46119552670368,36.66612257141649],[-4.461202881311809,36.66611464417448],[-4.461188098074032,36.66610581957127]]]}},{'type':'Feature','properties':{'area':'G2','block':'0,-1'},'geometry':{'type':'Polygon','coordinates':[[[-4.461180743465903,36.666113746813274],[-4.461173388857772,36.66612167405528],[-4.461188172095549,36.66613049865849],[-4.46119552670368,36.66612257141649],[-4.461180743465903,36.666113746813274]]]}},{'type':'Feature','properties':{'area':'G2','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.461173388857772,36.66612167405528],[-4.461166034249643,36.666129601297285],[-4.46118081748742,36.66613842590049],[-4.461188172095549,36.66613049865849],[-4.461173388857772,36.66612167405528]]]}},{'type':'Feature','properties':{'area':'G2','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.461166034249643,36.666129601297285],[-4.461158679641512,36.66613752853929],[-4.461173462879289,36.6661463531425],[-4.46118081748742,36.66613842590049],[-4.461166034249643,36.666129601297285]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.461285904003186,36.666104245877484],[-4.461275765106627,36.666098633165966],[-4.461265298160928,36.66611079857],[-4.4612754370574885,36.66611641128153],[-4.461285904003186,36.666104245877484]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.461275765106627,36.666098633165966],[-4.461265626210066,36.66609302045444],[-4.461255159264368,36.666105185858484],[-4.461265298160928,36.66611079857],[-4.461275765106627,36.666098633165966]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.461265626210066,36.66609302045444],[-4.4612554873135055,36.66608740774292],[-4.461245020367808,36.66609957314696],[-4.461255159264368,36.666105185858484],[-4.461265626210066,36.66609302045444]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-3'},'geometry':{'type':'Polygon','coordinates':[[[-4.461326787638565,36.66610891860801],[-4.461316648742005,36.666103305896485],[-4.4613061817963064,36.66611547130053],[-4.461316320692867,36.666121084012055],[-4.461326787638565,36.66610891860801]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-2'},'geometry':{'type':'Polygon','coordinates':[[[-4.461316648742005,36.666103305896485],[-4.4613065098454445,36.666097693184966],[-4.461296042899747,36.66610985858901],[-4.4613061817963064,36.66611547130053],[-4.461316648742005,36.666103305896485]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-1'},'geometry':{'type':'Polygon','coordinates':[[[-4.4613065098454445,36.666097693184966],[-4.461296370948884,36.66609208047344],[-4.461285904003186,36.666104245877484],[-4.461296042899747,36.66610985858901],[-4.4613065098454445,36.666097693184966]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.461296370948884,36.66609208047344],[-4.461286232052324,36.66608646776192],[-4.461275765106627,36.666098633165966],[-4.461285904003186,36.666104245877484],[-4.461296370948884,36.66609208047344]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.461286232052324,36.66608646776192],[-4.461276093155764,36.666080855050396],[-4.461265626210066,36.66609302045444],[-4.461275765106627,36.666098633165966],[-4.461286232052324,36.66608646776192]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.461276093155764,36.666080855050396],[-4.461265954259204,36.66607524233888],[-4.4612554873135055,36.66608740774292],[-4.461265626210066,36.66609302045444],[-4.461276093155764,36.666080855050396]]]}}]}</t>
+          <t>{'type':'FeatureCollection','features':[{'type':'Feature','properties':{'area':'G1','block':'-1,-3'},'geometry':{'type':'Polygon','coordinates':[[[-3.220742062578174,37.12749320120882],[-3.2207296688283997,37.12749320120882],[-3.2207296688283997,37.1275079825221],[-3.220742062578174,37.1275079825221],[-3.220742062578174,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,-2'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207296688283997,37.12749320120882],[-3.2207172750786257,37.12749320120882],[-3.2207172750786257,37.1275079825221],[-3.2207296688283997,37.1275079825221],[-3.2207296688283997,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,-1'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207172750786257,37.12749320120882],[-3.2207048813288512,37.12749320120882],[-3.2207048813288512,37.1275079825221],[-3.2207172750786257,37.1275079825221],[-3.2207172750786257,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,0'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207048813288512,37.12749320120882],[-3.2206924875790772,37.12749320120882],[-3.2206924875790772,37.1275079825221],[-3.2207048813288512,37.1275079825221],[-3.2207048813288512,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,1'},'geometry':{'type':'Polygon','coordinates':[[[-3.2206924875790772,37.12749320120882],[-3.2206800938293028,37.12749320120882],[-3.2206800938293028,37.1275079825221],[-3.2206924875790772,37.1275079825221],[-3.2206924875790772,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,2'},'geometry':{'type':'Polygon','coordinates':[[[-3.2206800938293028,37.12749320120882],[-3.2206677000795287,37.12749320120882],[-3.2206677000795287,37.1275079825221],[-3.2206800938293028,37.1275079825221],[-3.2206800938293028,37.12749320120882]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-3'},'geometry':{'type':'Polygon','coordinates':[[[-3.220742062578174,37.12747841989554],[-3.2207296688283997,37.12747841989554],[-3.2207296688283997,37.12749320120882],[-3.220742062578174,37.12749320120882],[-3.220742062578174,37.12747841989554]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-2'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207296688283997,37.12747841989554],[-3.2207172750786257,37.12747841989554],[-3.2207172750786257,37.12749320120882],[-3.2207296688283997,37.12749320120882],[-3.2207296688283997,37.12747841989554]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-3.2206924875790772,37.12747841989554],[-3.2206800938293028,37.12747841989554],[-3.2206800938293028,37.12749320120882],[-3.2206924875790772,37.12749320120882],[-3.2206924875790772,37.12747841989554]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-3.2206800938293028,37.12747841989554],[-3.2206677000795287,37.12747841989554],[-3.2206677000795287,37.12749320120882],[-3.2206800938293028,37.12749320120882],[-3.2206800938293028,37.12747841989554]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,-1'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207172750786257,37.12747841989554],[-3.2207048813288512,37.12747841989554],[-3.2207048813288512,37.12749320120882],[-3.2207172750786257,37.12749320120882],[-3.2207172750786257,37.12747841989554]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-3.2207048813288512,37.12747841989554],[-3.2206924875790772,37.12747841989554],[-3.2206924875790772,37.12749320120882],[-3.2207048813288512,37.12749320120882],[-3.2207048813288512,37.12747841989554]]]}}]}</t>
         </is>
       </c>
     </row>

</xml_diff>